<commit_message>
Update course plans and analysis documents for IKS and ISLL programs
- Modified various Excel files related to course analysis, including:
  - Färdighetskrav
  - Introfras
  - Nedlagda kursreferenser
  - Omfång på lärandemål
  - Samstämmighet svenska och engelska
  - Stavfel och språkbruk
  - Övrigt
  - Programkurser olänkade

- Updated markdown files for course plans (GLP29U, GLP2BQ, GLP2CX, GLP2NL, GLP2NN, GLP2VT, GLP2WP, GLP32S, LP1074, KLJMG) to reflect changes in quality notes and course requirements.

- Adjusted the number of quality notes in course plans and ensured consistency in references to courses that have been discontinued.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/03 IKS/Analys/Förkunskapskrav.xlsx
+++ b/vault-dalarna-university/03 IKS/Analys/Förkunskapskrav.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Förkunskapskrav" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$H$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$H$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -866,17 +866,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>GMN3EJ</t>
+          <t>GLP29U</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MPR</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2025-07-02</t>
+          <t>2019-06-17</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -887,34 +887,34 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>`Audioteknologi`</t>
+          <t>`Audioteknologi 2`</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>`LP1027` (nedlagd 2021-02-22); förkunskap nämner nedlagd kurs</t>
+          <t>`LP1080` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMN3EJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP29U</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>GMN3F2</t>
+          <t>GLP2BQ</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MPR</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>2019-10-09</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -925,34 +925,34 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>`Vetenskapsteori`</t>
+          <t>`Vetenskaplig uppsats i Ljud- och musikproduktion`</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>`GPG263` (nedlagd 2024-03-25); förkunskap nämner nedlagd kurs</t>
+          <t>`LP1065` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMN3F2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2BQ</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>GPA2P7</t>
+          <t>GLP2CX</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PEE</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2021-03-11</t>
+          <t>2020-01-31</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -963,34 +963,34 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>`Samhällsvetenskaplig metod och vetenskapsteori I`</t>
+          <t>`Audioteknologi 1`</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>`GPA32R` (nedlagd 2026-02-11); förkunskap nämner nedlagd kurs</t>
+          <t>`GLP2JZ` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPA2P7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2CX</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>GPA2R6</t>
+          <t>GLP2NL</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PEE</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2021-09-07</t>
+          <t>2021-03-12</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -1001,34 +1001,34 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>`Organisation - roller och intressenter`</t>
+          <t>`Vetenskaplig uppsats i Ljud- och musikproduktion`</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>`GPA356` (nedlagd 2026-02-11); förkunskap nämner nedlagd kurs</t>
+          <t>`LP1065` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPA2R6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2NL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GPA354</t>
+          <t>GLP2NN</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PEE</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2023-05-31</t>
+          <t>2021-03-12</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1039,34 +1039,34 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>`Arbetsrättens grunder`</t>
+          <t>`Vetenskaplig uppsats i Ljud- och musikproduktion`</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>`PA1021` (nedlagd 2026-02-11); förkunskap nämner nedlagd kurs</t>
+          <t>`LP1065` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPA354</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2NN</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>PA2009</t>
+          <t>GLP2VT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PEE</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2014-11-21</t>
+          <t>2022-03-11</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1077,34 +1077,34 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>`Samhällsvetenskaplig metod och vetenskapsteori I`</t>
+          <t>`Inspelning i studio`</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>`GPA32R` (nedlagd 2026-02-11); förkunskap nämner nedlagd kurs</t>
+          <t>`GLP29X` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PA2009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2VT</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>PA2010</t>
+          <t>GLP2VT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PEE</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2014-11-21</t>
+          <t>2022-03-11</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1115,34 +1115,34 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>`Samhällsvetenskaplig metod och vetenskapsteori I`</t>
+          <t>`Liveljud och liveinspelning`</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>`GPA32R` (nedlagd 2026-02-11); förkunskap nämner nedlagd kurs</t>
+          <t>`LP1064` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PA2010</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2VT</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>PA2011</t>
+          <t>GLP2VT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PEE</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2016-03-03</t>
+          <t>2022-03-11</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1153,34 +1153,34 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>`Samhällsvetenskaplig metod och vetenskapsteori I`</t>
+          <t>`Audioteknologi 2`</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>`GPA32R` (nedlagd 2026-02-11); förkunskap nämner nedlagd kurs</t>
+          <t>`LP1080` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PA2011</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2VT</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>APG275</t>
+          <t>GLP2WP</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PGA</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2021-10-06</t>
+          <t>2022-06-13</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1191,34 +1191,34 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>`Matematik 2a för grundlärare F-3`</t>
+          <t>`Inspelning i studio`</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>`MD2017` (nedlagd 2021-04-12); förkunskap nämner nedlagd kurs</t>
+          <t>`GLP29X` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG275</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2WP</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>APG275</t>
+          <t>GLP2WP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PGA</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2021-10-06</t>
+          <t>2022-06-13</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1229,34 +1229,34 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>`Matematik 2b för grundlärare F-3`</t>
+          <t>`Vetenskaplig uppsats i Ljud- och musikproduktion`</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>`MD2019` (nedlagd 2021-04-12); förkunskap nämner nedlagd kurs</t>
+          <t>`LP1065` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG275</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2WP</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>APG276</t>
+          <t>GLP32S</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PGA</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2021-10-06</t>
+          <t>2023-02-10</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1267,34 +1267,34 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>`Matematik 2a för grundlärare 4-6`</t>
+          <t>`Inspelning i studio`</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>`MD2016` (nedlagd 2022-08-29); förkunskap nämner nedlagd kurs</t>
+          <t>`GLP29X` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG276</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP32S</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>APG276</t>
+          <t>GLP32S</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PGA</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2021-10-06</t>
+          <t>2023-02-10</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1305,34 +1305,34 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>`Matematik 2b för grundlärare 4-6`</t>
+          <t>`Vetenskaplig uppsats i Ljud- och musikproduktion`</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>`MD2018` (nedlagd 2022-08-29); förkunskap nämner nedlagd kurs</t>
+          <t>`LP1065` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG276</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP32S</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>PG3025</t>
+          <t>LP1074</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PGA</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2013-07-03</t>
+          <t>2016-02-19</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1343,34 +1343,34 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>`Idrott`</t>
+          <t>`Inspelning i studio`</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>`IDB009` (nedlagd 2005-08-01); förkunskap nämner nedlagd kurs</t>
+          <t>`GLP29X` (nedlagd 2026-06-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PG3025</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=LP1074</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ARK25B</t>
+          <t>GMN3EJ</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>RKA</t>
+          <t>MPR</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2020-03-11</t>
+          <t>2025-07-02</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1381,34 +1381,34 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>`Vetenskapsteori`</t>
+          <t>`Audioteknologi`</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>`GPG263` (nedlagd 2024-03-25); förkunskap nämner nedlagd kurs</t>
+          <t>`LP1027` (nedlagd 2021-02-22); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK25B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMN3EJ</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ARK25C</t>
+          <t>GMN3F2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>RKA</t>
+          <t>MPR</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2020-03-11</t>
+          <t>2025-02-24</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1429,24 +1429,24 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK25C</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMN3F2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ARK29H</t>
+          <t>GPA2P7</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>RKA</t>
+          <t>PEE</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2023-09-08</t>
+          <t>2021-03-11</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1457,34 +1457,34 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>`Religionsvetenskap III`</t>
+          <t>`Samhällsvetenskaplig metod och vetenskapsteori I`</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>`GRK25S` (nedlagd 2023-03-01); förkunskap nämner nedlagd kurs</t>
+          <t>`GPA32R` (nedlagd 2026-02-11); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK29H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPA2P7</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ARK29J</t>
+          <t>GPA2R6</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>RKA</t>
+          <t>PEE</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2023-09-08</t>
+          <t>2021-09-07</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1495,34 +1495,34 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>`Religionsvetenskap III`</t>
+          <t>`Organisation - roller och intressenter`</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>`GRK25S` (nedlagd 2023-03-01); förkunskap nämner nedlagd kurs</t>
+          <t>`GPA356` (nedlagd 2026-02-11); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK29J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPA2R6</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GRK2R7</t>
+          <t>GPA354</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>RKA</t>
+          <t>PEE</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2021-09-07</t>
+          <t>2023-05-31</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1533,34 +1533,34 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>`Religionsvetenskap III`</t>
+          <t>`Arbetsrättens grunder`</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>`GRK25S` (nedlagd 2023-03-01); förkunskap nämner nedlagd kurs</t>
+          <t>`PA1021` (nedlagd 2026-02-11); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRK2R7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPA354</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GRK2R8</t>
+          <t>PA2009</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>RKA</t>
+          <t>PEE</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2021-09-07</t>
+          <t>2014-11-21</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1571,34 +1571,34 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>`Religionsvetenskap III`</t>
+          <t>`Samhällsvetenskaplig metod och vetenskapsteori I`</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>`GRK25S` (nedlagd 2023-03-01); förkunskap nämner nedlagd kurs</t>
+          <t>`GPA32R` (nedlagd 2026-02-11); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRK2R8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PA2009</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>RK3043</t>
+          <t>PA2010</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>RKA</t>
+          <t>PEE</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2014-09-19</t>
+          <t>2014-11-21</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1609,34 +1609,34 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>`Religionsvetenskap III`</t>
+          <t>`Samhällsvetenskaplig metod och vetenskapsteori I`</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>`GRK25S` (nedlagd 2023-03-01); förkunskap nämner nedlagd kurs</t>
+          <t>`GPA32R` (nedlagd 2026-02-11); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RK3043</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PA2010</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GRV266</t>
+          <t>PA2011</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>RVA</t>
+          <t>PEE</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2019-02-21</t>
+          <t>2016-03-03</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1647,34 +1647,34 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>`Extern redovisning`</t>
+          <t>`Samhällsvetenskaplig metod och vetenskapsteori I`</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>`FÖ1004` (nedlagd 2016-01-18); förkunskap nämner nedlagd kurs</t>
+          <t>`GPA32R` (nedlagd 2026-02-11); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRV266</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PA2011</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>RV1003</t>
+          <t>APG275</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>RVA</t>
+          <t>PGA</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2007-01-10</t>
+          <t>2021-10-06</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1685,34 +1685,34 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>`Extern redovisning`</t>
+          <t>`Matematik 2a för grundlärare F-3`</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>`FÖ1004` (nedlagd 2016-01-18); förkunskap nämner nedlagd kurs</t>
+          <t>`MD2017` (nedlagd 2021-04-12); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG275</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>RV1055</t>
+          <t>APG275</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>RVA</t>
+          <t>PGA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2016-03-03</t>
+          <t>2021-10-06</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1723,22 +1723,516 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
+          <t>`Matematik 2b för grundlärare F-3`</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>`MD2019` (nedlagd 2021-04-12); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG275</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>APG276</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PGA</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2021-10-06</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>`Matematik 2a för grundlärare 4-6`</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>`MD2016` (nedlagd 2022-08-29); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG276</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>APG276</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>PGA</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2021-10-06</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>`Matematik 2b för grundlärare 4-6`</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>`MD2018` (nedlagd 2022-08-29); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG276</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>PG3025</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>PGA</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2013-07-03</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>`Idrott`</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>`IDB009` (nedlagd 2005-08-01); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PG3025</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>ARK25B</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>RKA</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2020-03-11</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>`Vetenskapsteori`</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>`GPG263` (nedlagd 2024-03-25); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK25B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>ARK25C</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>RKA</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2020-03-11</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>`Vetenskapsteori`</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>`GPG263` (nedlagd 2024-03-25); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK25C</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>ARK29H</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>RKA</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2023-09-08</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>`Religionsvetenskap III`</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>`GRK25S` (nedlagd 2023-03-01); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK29H</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>ARK29J</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>RKA</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2023-09-08</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>`Religionsvetenskap III`</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>`GRK25S` (nedlagd 2023-03-01); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK29J</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>GRK2R7</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>RKA</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2021-09-07</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>`Religionsvetenskap III`</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>`GRK25S` (nedlagd 2023-03-01); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRK2R7</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>GRK2R8</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>RKA</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2021-09-07</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>`Religionsvetenskap III`</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>`GRK25S` (nedlagd 2023-03-01); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRK2R8</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>RK3043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>RKA</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2014-09-19</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>`Religionsvetenskap III`</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>`GRK25S` (nedlagd 2023-03-01); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RK3043</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>GRV266</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>RVA</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2019-02-21</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>`Extern redovisning`</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>`FÖ1004` (nedlagd 2016-01-18); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRV266</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>RV1003</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>RVA</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2007-01-10</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>`Extern redovisning`</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>`FÖ1004` (nedlagd 2016-01-18); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1003</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>RV1055</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>RVA</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2016-03-03</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
           <t>`Perspektiv på företagande`</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>`FÖ1057` (nedlagd 2021-02-15); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1055</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H34"/>
+  <autoFilter ref="A1:H47"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
@@ -1806,6 +2300,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId92"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>